<commit_message>
Added dashboard charts and UI improvements
</commit_message>
<xml_diff>
--- a/companies.xlsx
+++ b/companies.xlsx
@@ -440,7 +440,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -454,77 +454,77 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t xml:space="preserve">India </t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>United States</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>India</t>
+          <t xml:space="preserve"> USA</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t xml:space="preserve"> Technology</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>usa</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>Infosys</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -534,17 +534,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>India</t>
+          <t xml:space="preserve">INDIA </t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t xml:space="preserve">Google </t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -554,7 +554,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>USA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated API URL and CORS
</commit_message>
<xml_diff>
--- a/companies.xlsx
+++ b/companies.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,6 +558,26 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>12</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>tcs</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>It</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Usa</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>